<commit_message>
Add rubrica rule management and comparison workflow
</commit_message>
<xml_diff>
--- a/scripts/01. Tabela de Natureza de Rubricas..xlsx
+++ b/scripts/01. Tabela de Natureza de Rubricas..xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1OD650nFufniPR7CJNVrJNCb_pI70Jjm2\VISITOR\VISITOR PROJETOS\PROJETO RUBRICAS\TABELAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5902039B-BEE3-40AF-9989-0CC873D2F7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF18454A-2038-4776-A9D2-9C35FFEEC0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62667083-EF7A-4441-AE58-07703D1210CF}"/>
   </bookViews>
@@ -1167,6 +1167,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1196,8 +1199,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1538,8 +1542,8 @@
     <col min="1" max="1" width="6.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1573,9 +1577,10 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
-        <v>41640</v>
-      </c>
+      <c r="D2" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -1587,9 +1592,10 @@
       <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
-        <v>41640</v>
-      </c>
+      <c r="D3" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -1601,10 +1607,10 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="D4">
-        <v>41640</v>
-      </c>
-      <c r="E4">
+      <c r="D4" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E4" s="1">
         <v>45412</v>
       </c>
     </row>
@@ -1618,9 +1624,10 @@
       <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="D5">
-        <v>41640</v>
-      </c>
+      <c r="D5" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -1632,9 +1639,10 @@
       <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="D6">
-        <v>41640</v>
-      </c>
+      <c r="D6" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -1646,9 +1654,10 @@
       <c r="C7" t="s">
         <v>17</v>
       </c>
-      <c r="D7">
-        <v>41640</v>
-      </c>
+      <c r="D7" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -1660,9 +1669,10 @@
       <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="D8">
-        <v>41640</v>
-      </c>
+      <c r="D8" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -1674,9 +1684,10 @@
       <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9">
-        <v>41640</v>
-      </c>
+      <c r="D9" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -1688,9 +1699,10 @@
       <c r="C10" t="s">
         <v>23</v>
       </c>
-      <c r="D10">
-        <v>41640</v>
-      </c>
+      <c r="D10" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -1702,9 +1714,10 @@
       <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11">
-        <v>41640</v>
-      </c>
+      <c r="D11" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -1716,9 +1729,10 @@
       <c r="C12" t="s">
         <v>27</v>
       </c>
-      <c r="D12">
-        <v>41640</v>
-      </c>
+      <c r="D12" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -1730,9 +1744,10 @@
       <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13">
-        <v>41640</v>
-      </c>
+      <c r="D13" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -1744,9 +1759,10 @@
       <c r="C14" t="s">
         <v>31</v>
       </c>
-      <c r="D14">
-        <v>41640</v>
-      </c>
+      <c r="D14" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -1758,10 +1774,10 @@
       <c r="C15" t="s">
         <v>33</v>
       </c>
-      <c r="D15">
-        <v>41640</v>
-      </c>
-      <c r="E15">
+      <c r="D15" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E15" s="1">
         <v>46022</v>
       </c>
     </row>
@@ -1775,9 +1791,10 @@
       <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="1">
         <v>46023</v>
       </c>
+      <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
@@ -1789,10 +1806,10 @@
       <c r="C17" t="s">
         <v>36</v>
       </c>
-      <c r="D17">
-        <v>41640</v>
-      </c>
-      <c r="E17">
+      <c r="D17" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E17" s="1">
         <v>46022</v>
       </c>
     </row>
@@ -1806,9 +1823,10 @@
       <c r="C18" t="s">
         <v>37</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <v>46024</v>
       </c>
+      <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
@@ -1820,9 +1838,10 @@
       <c r="C19" t="s">
         <v>39</v>
       </c>
-      <c r="D19">
-        <v>41640</v>
-      </c>
+      <c r="D19" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
@@ -1834,9 +1853,10 @@
       <c r="C20" t="s">
         <v>40</v>
       </c>
-      <c r="D20">
-        <v>41640</v>
-      </c>
+      <c r="D20" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E20" s="1"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
@@ -1848,10 +1868,10 @@
       <c r="C21" t="s">
         <v>42</v>
       </c>
-      <c r="D21">
-        <v>41640</v>
-      </c>
-      <c r="E21">
+      <c r="D21" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E21" s="1">
         <v>45046</v>
       </c>
     </row>
@@ -1865,10 +1885,10 @@
       <c r="C22" t="s">
         <v>39</v>
       </c>
-      <c r="D22">
-        <v>41640</v>
-      </c>
-      <c r="E22">
+      <c r="D22" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E22" s="1">
         <v>45046</v>
       </c>
     </row>
@@ -1882,9 +1902,10 @@
       <c r="C23" t="s">
         <v>43</v>
       </c>
-      <c r="D23">
-        <v>41640</v>
-      </c>
+      <c r="D23" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E23" s="1"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -1896,9 +1917,10 @@
       <c r="C24" t="s">
         <v>45</v>
       </c>
-      <c r="D24">
-        <v>41640</v>
-      </c>
+      <c r="D24" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E24" s="1"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -1910,9 +1932,10 @@
       <c r="C25" t="s">
         <v>46</v>
       </c>
-      <c r="D25">
-        <v>41640</v>
-      </c>
+      <c r="D25" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E25" s="1"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -1924,9 +1947,10 @@
       <c r="C26" t="s">
         <v>48</v>
       </c>
-      <c r="D26">
-        <v>41640</v>
-      </c>
+      <c r="D26" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
@@ -1938,9 +1962,10 @@
       <c r="C27" t="s">
         <v>49</v>
       </c>
-      <c r="D27">
-        <v>41640</v>
-      </c>
+      <c r="D27" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E27" s="1"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
@@ -1952,9 +1977,10 @@
       <c r="C28" t="s">
         <v>51</v>
       </c>
-      <c r="D28">
-        <v>41640</v>
-      </c>
+      <c r="D28" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E28" s="1"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
@@ -1966,9 +1992,10 @@
       <c r="C29" t="s">
         <v>53</v>
       </c>
-      <c r="D29">
-        <v>41640</v>
-      </c>
+      <c r="D29" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E29" s="1"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
@@ -1980,9 +2007,10 @@
       <c r="C30" t="s">
         <v>55</v>
       </c>
-      <c r="D30">
-        <v>41640</v>
-      </c>
+      <c r="D30" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E30" s="1"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
@@ -1994,9 +2022,10 @@
       <c r="C31" t="s">
         <v>57</v>
       </c>
-      <c r="D31">
-        <v>41640</v>
-      </c>
+      <c r="D31" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E31" s="1"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
@@ -2008,11 +2037,12 @@
       <c r="C32" t="s">
         <v>59</v>
       </c>
-      <c r="D32">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D32" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>1203</v>
       </c>
@@ -2022,11 +2052,12 @@
       <c r="C33" t="s">
         <v>61</v>
       </c>
-      <c r="D33">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D33" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>1204</v>
       </c>
@@ -2036,11 +2067,12 @@
       <c r="C34" t="s">
         <v>63</v>
       </c>
-      <c r="D34">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D34" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>1205</v>
       </c>
@@ -2050,11 +2082,12 @@
       <c r="C35" t="s">
         <v>65</v>
       </c>
-      <c r="D35">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D35" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>1206</v>
       </c>
@@ -2064,11 +2097,12 @@
       <c r="C36" t="s">
         <v>67</v>
       </c>
-      <c r="D36">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D36" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E36" s="1"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>1207</v>
       </c>
@@ -2078,11 +2112,12 @@
       <c r="C37" t="s">
         <v>68</v>
       </c>
-      <c r="D37">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D37" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E37" s="1"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>1208</v>
       </c>
@@ -2092,11 +2127,12 @@
       <c r="C38" t="s">
         <v>70</v>
       </c>
-      <c r="D38">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D38" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>1209</v>
       </c>
@@ -2106,11 +2142,12 @@
       <c r="C39" t="s">
         <v>72</v>
       </c>
-      <c r="D39">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D39" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E39" s="1"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>1210</v>
       </c>
@@ -2120,11 +2157,12 @@
       <c r="C40" t="s">
         <v>74</v>
       </c>
-      <c r="D40">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D40" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E40" s="1"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>1211</v>
       </c>
@@ -2134,11 +2172,12 @@
       <c r="C41" t="s">
         <v>76</v>
       </c>
-      <c r="D41">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D41" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E41" s="1"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>1212</v>
       </c>
@@ -2148,11 +2187,12 @@
       <c r="C42" t="s">
         <v>78</v>
       </c>
-      <c r="D42">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D42" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E42" s="1"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>1213</v>
       </c>
@@ -2162,11 +2202,12 @@
       <c r="C43" t="s">
         <v>79</v>
       </c>
-      <c r="D43">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D43" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E43" s="1"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>1214</v>
       </c>
@@ -2176,11 +2217,12 @@
       <c r="C44" t="s">
         <v>81</v>
       </c>
-      <c r="D44">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D44" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E44" s="1"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>1215</v>
       </c>
@@ -2190,11 +2232,12 @@
       <c r="C45" t="s">
         <v>83</v>
       </c>
-      <c r="D45">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D45" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E45" s="1"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>1216</v>
       </c>
@@ -2204,11 +2247,12 @@
       <c r="C46" t="s">
         <v>84</v>
       </c>
-      <c r="D46">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D46" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E46" s="1"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>1217</v>
       </c>
@@ -2218,11 +2262,12 @@
       <c r="C47" t="s">
         <v>86</v>
       </c>
-      <c r="D47">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D47" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E47" s="1"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>1225</v>
       </c>
@@ -2232,11 +2277,12 @@
       <c r="C48" t="s">
         <v>88</v>
       </c>
-      <c r="D48">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D48" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E48" s="1"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>1230</v>
       </c>
@@ -2246,11 +2292,12 @@
       <c r="C49" t="s">
         <v>90</v>
       </c>
-      <c r="D49">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D49" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E49" s="1"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>1299</v>
       </c>
@@ -2260,11 +2307,12 @@
       <c r="C50" t="s">
         <v>92</v>
       </c>
-      <c r="D50">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D50" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E50" s="1"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>1300</v>
       </c>
@@ -2274,11 +2322,12 @@
       <c r="C51" t="s">
         <v>94</v>
       </c>
-      <c r="D51">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D51" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E51" s="1"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>1350</v>
       </c>
@@ -2288,11 +2337,12 @@
       <c r="C52" t="s">
         <v>96</v>
       </c>
-      <c r="D52">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D52" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E52" s="1"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>1351</v>
       </c>
@@ -2302,11 +2352,12 @@
       <c r="C53" t="s">
         <v>98</v>
       </c>
-      <c r="D53">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D53" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E53" s="1"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>1352</v>
       </c>
@@ -2316,11 +2367,12 @@
       <c r="C54" t="s">
         <v>100</v>
       </c>
-      <c r="D54">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D54" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E54" s="1"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>1401</v>
       </c>
@@ -2330,11 +2382,12 @@
       <c r="C55" t="s">
         <v>102</v>
       </c>
-      <c r="D55">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D55" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E55" s="1"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>1402</v>
       </c>
@@ -2344,11 +2397,12 @@
       <c r="C56" t="s">
         <v>104</v>
       </c>
-      <c r="D56">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D56" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E56" s="1"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>1403</v>
       </c>
@@ -2358,11 +2412,12 @@
       <c r="C57" t="s">
         <v>106</v>
       </c>
-      <c r="D57">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D57" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E57" s="1"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>1404</v>
       </c>
@@ -2372,11 +2427,12 @@
       <c r="C58" t="s">
         <v>108</v>
       </c>
-      <c r="D58">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D58" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E58" s="1"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>1405</v>
       </c>
@@ -2386,11 +2442,12 @@
       <c r="C59" t="s">
         <v>110</v>
       </c>
-      <c r="D59">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D59" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E59" s="1"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>1406</v>
       </c>
@@ -2400,11 +2457,12 @@
       <c r="C60" t="s">
         <v>112</v>
       </c>
-      <c r="D60">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D60" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E60" s="1"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>1407</v>
       </c>
@@ -2414,11 +2472,12 @@
       <c r="C61" t="s">
         <v>114</v>
       </c>
-      <c r="D61">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D61" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E61" s="1"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>1409</v>
       </c>
@@ -2428,11 +2487,12 @@
       <c r="C62" t="s">
         <v>115</v>
       </c>
-      <c r="D62">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D62" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E62" s="1"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>1410</v>
       </c>
@@ -2442,11 +2502,12 @@
       <c r="C63" t="s">
         <v>117</v>
       </c>
-      <c r="D63">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D63" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E63" s="1"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>1411</v>
       </c>
@@ -2456,9 +2517,10 @@
       <c r="C64" t="s">
         <v>119</v>
       </c>
-      <c r="D64">
-        <v>41640</v>
-      </c>
+      <c r="D64" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E64" s="1"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
@@ -2470,9 +2532,10 @@
       <c r="C65" t="s">
         <v>121</v>
       </c>
-      <c r="D65">
-        <v>41640</v>
-      </c>
+      <c r="D65" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E65" s="1"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
@@ -2484,9 +2547,10 @@
       <c r="C66" t="s">
         <v>123</v>
       </c>
-      <c r="D66">
-        <v>41640</v>
-      </c>
+      <c r="D66" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E66" s="1"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67">
@@ -2498,9 +2562,10 @@
       <c r="C67" t="s">
         <v>125</v>
       </c>
-      <c r="D67">
-        <v>41640</v>
-      </c>
+      <c r="D67" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E67" s="1"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68">
@@ -2512,10 +2577,10 @@
       <c r="C68" t="s">
         <v>127</v>
       </c>
-      <c r="D68">
+      <c r="D68" s="1">
         <v>43221</v>
       </c>
-      <c r="E68">
+      <c r="E68" s="1">
         <v>43555</v>
       </c>
     </row>
@@ -2529,9 +2594,10 @@
       <c r="C69" t="s">
         <v>128</v>
       </c>
-      <c r="D69">
+      <c r="D69" s="1">
         <v>43556</v>
       </c>
+      <c r="E69" s="1"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70">
@@ -2543,10 +2609,10 @@
       <c r="C70" t="s">
         <v>129</v>
       </c>
-      <c r="D70">
+      <c r="D70" s="1">
         <v>43221</v>
       </c>
-      <c r="E70">
+      <c r="E70" s="1">
         <v>43555</v>
       </c>
     </row>
@@ -2560,9 +2626,10 @@
       <c r="C71" t="s">
         <v>131</v>
       </c>
-      <c r="D71">
+      <c r="D71" s="1">
         <v>43922</v>
       </c>
+      <c r="E71" s="1"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72">
@@ -2574,9 +2641,10 @@
       <c r="C72" t="s">
         <v>133</v>
       </c>
-      <c r="D72">
-        <v>41640</v>
-      </c>
+      <c r="D72" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E72" s="1"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73">
@@ -2588,9 +2656,10 @@
       <c r="C73" t="s">
         <v>135</v>
       </c>
-      <c r="D73">
-        <v>41640</v>
-      </c>
+      <c r="D73" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E73" s="1"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74">
@@ -2602,9 +2671,10 @@
       <c r="C74" t="s">
         <v>137</v>
       </c>
-      <c r="D74">
-        <v>41640</v>
-      </c>
+      <c r="D74" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E74" s="1"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75">
@@ -2616,9 +2686,10 @@
       <c r="C75" t="s">
         <v>139</v>
       </c>
-      <c r="D75">
-        <v>41640</v>
-      </c>
+      <c r="D75" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E75" s="1"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76">
@@ -2630,9 +2701,10 @@
       <c r="C76" t="s">
         <v>141</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="1">
         <v>43221</v>
       </c>
+      <c r="E76" s="1"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77">
@@ -2644,10 +2716,10 @@
       <c r="C77" t="s">
         <v>142</v>
       </c>
-      <c r="D77">
-        <v>41640</v>
-      </c>
-      <c r="E77">
+      <c r="D77" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E77" s="1">
         <v>43220</v>
       </c>
     </row>
@@ -2661,10 +2733,10 @@
       <c r="C78" t="s">
         <v>144</v>
       </c>
-      <c r="D78">
-        <v>41640</v>
-      </c>
-      <c r="E78">
+      <c r="D78" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E78" s="1">
         <v>43220</v>
       </c>
     </row>
@@ -2678,9 +2750,10 @@
       <c r="C79" t="s">
         <v>146</v>
       </c>
-      <c r="D79">
-        <v>41640</v>
-      </c>
+      <c r="D79" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E79" s="1"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80">
@@ -2692,10 +2765,10 @@
       <c r="C80" t="s">
         <v>148</v>
       </c>
-      <c r="D80">
-        <v>41640</v>
-      </c>
-      <c r="E80">
+      <c r="D80" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E80" s="1">
         <v>46022</v>
       </c>
     </row>
@@ -2709,9 +2782,10 @@
       <c r="C81" t="s">
         <v>149</v>
       </c>
-      <c r="D81">
+      <c r="D81" s="1">
         <v>46025</v>
       </c>
+      <c r="E81" s="1"/>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82">
@@ -2723,10 +2797,10 @@
       <c r="C82" t="s">
         <v>150</v>
       </c>
-      <c r="D82">
-        <v>41640</v>
-      </c>
-      <c r="E82">
+      <c r="D82" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E82" s="1">
         <v>44377</v>
       </c>
     </row>
@@ -2740,9 +2814,10 @@
       <c r="C83" t="s">
         <v>152</v>
       </c>
-      <c r="D83">
-        <v>41640</v>
-      </c>
+      <c r="D83" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E83" s="1"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84">
@@ -2754,9 +2829,10 @@
       <c r="C84" t="s">
         <v>153</v>
       </c>
-      <c r="D84">
-        <v>41640</v>
-      </c>
+      <c r="D84" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E84" s="1"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85">
@@ -2768,9 +2844,10 @@
       <c r="C85" t="s">
         <v>154</v>
       </c>
-      <c r="D85">
-        <v>41640</v>
-      </c>
+      <c r="D85" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E85" s="1"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86">
@@ -2782,9 +2859,10 @@
       <c r="C86" t="s">
         <v>155</v>
       </c>
-      <c r="D86">
-        <v>41640</v>
-      </c>
+      <c r="D86" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E86" s="1"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87">
@@ -2796,9 +2874,10 @@
       <c r="C87" t="s">
         <v>156</v>
       </c>
-      <c r="D87">
-        <v>41640</v>
-      </c>
+      <c r="D87" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E87" s="1"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88">
@@ -2810,9 +2889,10 @@
       <c r="C88" t="s">
         <v>157</v>
       </c>
-      <c r="D88">
-        <v>41640</v>
-      </c>
+      <c r="D88" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E88" s="1"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89">
@@ -2824,10 +2904,10 @@
       <c r="C89" t="s">
         <v>158</v>
       </c>
-      <c r="D89">
-        <v>41640</v>
-      </c>
-      <c r="E89">
+      <c r="D89" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E89" s="1">
         <v>46022</v>
       </c>
     </row>
@@ -2841,9 +2921,10 @@
       <c r="C90" t="s">
         <v>160</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="1">
         <v>46026</v>
       </c>
+      <c r="E90" s="1"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91">
@@ -2855,9 +2936,10 @@
       <c r="C91" t="s">
         <v>162</v>
       </c>
-      <c r="D91">
-        <v>41640</v>
-      </c>
+      <c r="D91" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E91" s="1"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92">
@@ -2869,9 +2951,10 @@
       <c r="C92" t="s">
         <v>163</v>
       </c>
-      <c r="D92">
-        <v>41640</v>
-      </c>
+      <c r="D92" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E92" s="1"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93">
@@ -2883,9 +2966,10 @@
       <c r="C93" t="s">
         <v>165</v>
       </c>
-      <c r="D93">
-        <v>41640</v>
-      </c>
+      <c r="D93" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E93" s="1"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94">
@@ -2897,10 +2981,10 @@
       <c r="C94" t="s">
         <v>166</v>
       </c>
-      <c r="D94">
-        <v>41640</v>
-      </c>
-      <c r="E94">
+      <c r="D94" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E94" s="1">
         <v>43220</v>
       </c>
     </row>
@@ -2914,10 +2998,10 @@
       <c r="C95" t="s">
         <v>168</v>
       </c>
-      <c r="D95">
+      <c r="D95" s="1">
         <v>43221</v>
       </c>
-      <c r="E95">
+      <c r="E95" s="1">
         <v>43555</v>
       </c>
     </row>
@@ -2931,9 +3015,10 @@
       <c r="C96" t="s">
         <v>169</v>
       </c>
-      <c r="D96">
+      <c r="D96" s="1">
         <v>43556</v>
       </c>
+      <c r="E96" s="1"/>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97">
@@ -2945,10 +3030,10 @@
       <c r="C97" t="s">
         <v>170</v>
       </c>
-      <c r="D97">
+      <c r="D97" s="1">
         <v>43221</v>
       </c>
-      <c r="E97">
+      <c r="E97" s="1">
         <v>43555</v>
       </c>
     </row>
@@ -2962,9 +3047,10 @@
       <c r="C98" t="s">
         <v>172</v>
       </c>
-      <c r="D98">
-        <v>41640</v>
-      </c>
+      <c r="D98" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E98" s="1"/>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99">
@@ -2976,9 +3062,10 @@
       <c r="C99" t="s">
         <v>174</v>
       </c>
-      <c r="D99">
-        <v>41640</v>
-      </c>
+      <c r="D99" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E99" s="1"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100">
@@ -2990,9 +3077,10 @@
       <c r="C100" t="s">
         <v>176</v>
       </c>
-      <c r="D100">
-        <v>41640</v>
-      </c>
+      <c r="D100" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E100" s="1"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101">
@@ -3004,10 +3092,10 @@
       <c r="C101" t="s">
         <v>178</v>
       </c>
-      <c r="D101">
-        <v>41640</v>
-      </c>
-      <c r="E101">
+      <c r="D101" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E101" s="1">
         <v>44408</v>
       </c>
     </row>
@@ -3021,9 +3109,10 @@
       <c r="C102" t="s">
         <v>179</v>
       </c>
-      <c r="D102">
-        <v>41640</v>
-      </c>
+      <c r="D102" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E102" s="1"/>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103">
@@ -3035,10 +3124,10 @@
       <c r="C103" t="s">
         <v>181</v>
       </c>
-      <c r="D103">
-        <v>41640</v>
-      </c>
-      <c r="E103">
+      <c r="D103" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E103" s="1">
         <v>44408</v>
       </c>
     </row>
@@ -3052,9 +3141,10 @@
       <c r="C104" t="s">
         <v>183</v>
       </c>
-      <c r="D104">
-        <v>41640</v>
-      </c>
+      <c r="D104" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E104" s="1"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105">
@@ -3066,9 +3156,10 @@
       <c r="C105" t="s">
         <v>184</v>
       </c>
-      <c r="D105">
-        <v>41640</v>
-      </c>
+      <c r="D105" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E105" s="1"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106">
@@ -3080,9 +3171,10 @@
       <c r="C106" t="s">
         <v>186</v>
       </c>
-      <c r="D106">
-        <v>41640</v>
-      </c>
+      <c r="D106" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E106" s="1"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107">
@@ -3094,9 +3186,10 @@
       <c r="C107" t="s">
         <v>188</v>
       </c>
-      <c r="D107">
-        <v>41640</v>
-      </c>
+      <c r="D107" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E107" s="1"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108">
@@ -3108,9 +3201,10 @@
       <c r="C108" t="s">
         <v>189</v>
       </c>
-      <c r="D108">
-        <v>41640</v>
-      </c>
+      <c r="D108" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E108" s="1"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109">
@@ -3122,9 +3216,10 @@
       <c r="C109" t="s">
         <v>190</v>
       </c>
-      <c r="D109">
-        <v>41640</v>
-      </c>
+      <c r="D109" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E109" s="1"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110">
@@ -3136,9 +3231,10 @@
       <c r="C110" t="s">
         <v>192</v>
       </c>
-      <c r="D110">
-        <v>41640</v>
-      </c>
+      <c r="D110" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E110" s="1"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111">
@@ -3150,9 +3246,10 @@
       <c r="C111" t="s">
         <v>194</v>
       </c>
-      <c r="D111">
-        <v>41640</v>
-      </c>
+      <c r="D111" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E111" s="1"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112">
@@ -3164,11 +3261,12 @@
       <c r="C112" t="s">
         <v>196</v>
       </c>
-      <c r="D112">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D112" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E112" s="1"/>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>3520</v>
       </c>
@@ -3178,11 +3276,12 @@
       <c r="C113" t="s">
         <v>198</v>
       </c>
-      <c r="D113">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D113" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E113" s="1"/>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>3525</v>
       </c>
@@ -3192,11 +3291,12 @@
       <c r="C114" t="s">
         <v>200</v>
       </c>
-      <c r="D114">
+      <c r="D114" s="1">
         <v>43221</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E114" s="1"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>4010</v>
       </c>
@@ -3206,11 +3306,12 @@
       <c r="C115" t="s">
         <v>202</v>
       </c>
-      <c r="D115">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D115" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E115" s="1"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>4011</v>
       </c>
@@ -3220,11 +3321,12 @@
       <c r="C116" t="s">
         <v>204</v>
       </c>
-      <c r="D116">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D116" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E116" s="1"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>4050</v>
       </c>
@@ -3234,11 +3336,12 @@
       <c r="C117" t="s">
         <v>206</v>
       </c>
-      <c r="D117">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D117" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E117" s="1"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>4051</v>
       </c>
@@ -3248,11 +3351,12 @@
       <c r="C118" t="s">
         <v>208</v>
       </c>
-      <c r="D118">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D118" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E118" s="1"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>5001</v>
       </c>
@@ -3262,11 +3366,12 @@
       <c r="C119" t="s">
         <v>210</v>
       </c>
-      <c r="D119">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D119" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E119" s="1"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>5005</v>
       </c>
@@ -3276,11 +3381,12 @@
       <c r="C120" t="s">
         <v>212</v>
       </c>
-      <c r="D120">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D120" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E120" s="1"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>5501</v>
       </c>
@@ -3290,11 +3396,12 @@
       <c r="C121" t="s">
         <v>214</v>
       </c>
-      <c r="D121">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D121" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E121" s="1"/>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>5504</v>
       </c>
@@ -3304,11 +3411,12 @@
       <c r="C122" t="s">
         <v>216</v>
       </c>
-      <c r="D122">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D122" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E122" s="1"/>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>5510</v>
       </c>
@@ -3318,11 +3426,12 @@
       <c r="C123" t="s">
         <v>218</v>
       </c>
-      <c r="D123">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D123" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E123" s="1"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>6000</v>
       </c>
@@ -3332,11 +3441,12 @@
       <c r="C124" t="s">
         <v>220</v>
       </c>
-      <c r="D124">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D124" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E124" s="1"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>6001</v>
       </c>
@@ -3346,11 +3456,12 @@
       <c r="C125" t="s">
         <v>222</v>
       </c>
-      <c r="D125">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D125" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E125" s="1"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>6002</v>
       </c>
@@ -3360,11 +3471,12 @@
       <c r="C126" t="s">
         <v>224</v>
       </c>
-      <c r="D126">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D126" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E126" s="1"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>6003</v>
       </c>
@@ -3374,11 +3486,12 @@
       <c r="C127" t="s">
         <v>226</v>
       </c>
-      <c r="D127">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D127" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E127" s="1"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>6004</v>
       </c>
@@ -3388,11 +3501,12 @@
       <c r="C128" t="s">
         <v>227</v>
       </c>
-      <c r="D128">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D128" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E128" s="1"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>6006</v>
       </c>
@@ -3402,11 +3516,12 @@
       <c r="C129" t="s">
         <v>229</v>
       </c>
-      <c r="D129">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D129" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E129" s="1"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>6007</v>
       </c>
@@ -3416,11 +3531,12 @@
       <c r="C130" t="s">
         <v>230</v>
       </c>
-      <c r="D130">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D130" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E130" s="1"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>6101</v>
       </c>
@@ -3430,11 +3546,12 @@
       <c r="C131" t="s">
         <v>232</v>
       </c>
-      <c r="D131">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D131" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E131" s="1"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>6102</v>
       </c>
@@ -3444,11 +3561,12 @@
       <c r="C132" t="s">
         <v>234</v>
       </c>
-      <c r="D132">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D132" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E132" s="1"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>6103</v>
       </c>
@@ -3458,11 +3576,12 @@
       <c r="C133" t="s">
         <v>236</v>
       </c>
-      <c r="D133">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D133" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E133" s="1"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>6104</v>
       </c>
@@ -3472,11 +3591,12 @@
       <c r="C134" t="s">
         <v>238</v>
       </c>
-      <c r="D134">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D134" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E134" s="1"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>6105</v>
       </c>
@@ -3486,11 +3606,12 @@
       <c r="C135" t="s">
         <v>240</v>
       </c>
-      <c r="D135">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D135" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E135" s="1"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>6106</v>
       </c>
@@ -3500,11 +3621,12 @@
       <c r="C136" t="s">
         <v>242</v>
       </c>
-      <c r="D136">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D136" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E136" s="1"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>6107</v>
       </c>
@@ -3514,11 +3636,12 @@
       <c r="C137" t="s">
         <v>244</v>
       </c>
-      <c r="D137">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D137" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E137" s="1"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>6108</v>
       </c>
@@ -3528,11 +3651,12 @@
       <c r="C138" t="s">
         <v>246</v>
       </c>
-      <c r="D138">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D138" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E138" s="1"/>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>6119</v>
       </c>
@@ -3542,11 +3666,12 @@
       <c r="C139" t="s">
         <v>248</v>
       </c>
-      <c r="D139">
+      <c r="D139" s="1">
         <v>43922</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E139" s="1"/>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>6129</v>
       </c>
@@ -3556,11 +3681,12 @@
       <c r="C140" t="s">
         <v>250</v>
       </c>
-      <c r="D140">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D140" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E140" s="1"/>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>6901</v>
       </c>
@@ -3570,11 +3696,12 @@
       <c r="C141" t="s">
         <v>252</v>
       </c>
-      <c r="D141">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D141" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E141" s="1"/>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>6904</v>
       </c>
@@ -3584,11 +3711,12 @@
       <c r="C142" t="s">
         <v>254</v>
       </c>
-      <c r="D142">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D142" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E142" s="1"/>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>7001</v>
       </c>
@@ -3598,11 +3726,12 @@
       <c r="C143" t="s">
         <v>256</v>
       </c>
-      <c r="D143">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D143" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E143" s="1"/>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>7002</v>
       </c>
@@ -3612,11 +3741,12 @@
       <c r="C144" t="s">
         <v>258</v>
       </c>
-      <c r="D144">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D144" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E144" s="1"/>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>7003</v>
       </c>
@@ -3626,11 +3756,12 @@
       <c r="C145" t="s">
         <v>260</v>
       </c>
-      <c r="D145">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D145" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E145" s="1"/>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>7004</v>
       </c>
@@ -3640,11 +3771,12 @@
       <c r="C146" t="s">
         <v>261</v>
       </c>
-      <c r="D146">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D146" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E146" s="1"/>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>7005</v>
       </c>
@@ -3654,11 +3786,12 @@
       <c r="C147" t="s">
         <v>263</v>
       </c>
-      <c r="D147">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D147" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E147" s="1"/>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>7006</v>
       </c>
@@ -3668,11 +3801,12 @@
       <c r="C148" t="s">
         <v>265</v>
       </c>
-      <c r="D148">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D148" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E148" s="1"/>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>7007</v>
       </c>
@@ -3682,11 +3816,12 @@
       <c r="C149" t="s">
         <v>267</v>
       </c>
-      <c r="D149">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D149" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E149" s="1"/>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>7008</v>
       </c>
@@ -3696,11 +3831,12 @@
       <c r="C150" t="s">
         <v>269</v>
       </c>
-      <c r="D150">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D150" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E150" s="1"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>9200</v>
       </c>
@@ -3710,11 +3846,12 @@
       <c r="C151" t="s">
         <v>271</v>
       </c>
-      <c r="D151">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D151" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E151" s="1"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>9201</v>
       </c>
@@ -3724,11 +3861,12 @@
       <c r="C152" t="s">
         <v>273</v>
       </c>
-      <c r="D152">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D152" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E152" s="1"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>9202</v>
       </c>
@@ -3738,11 +3876,12 @@
       <c r="C153" t="s">
         <v>275</v>
       </c>
-      <c r="D153">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D153" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E153" s="1"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>9203</v>
       </c>
@@ -3752,11 +3891,12 @@
       <c r="C154" t="s">
         <v>276</v>
       </c>
-      <c r="D154">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D154" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E154" s="1"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>9205</v>
       </c>
@@ -3766,11 +3906,12 @@
       <c r="C155" t="s">
         <v>278</v>
       </c>
-      <c r="D155">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D155" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E155" s="1"/>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>9207</v>
       </c>
@@ -3780,11 +3921,12 @@
       <c r="C156" t="s">
         <v>280</v>
       </c>
-      <c r="D156">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D156" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E156" s="1"/>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>9208</v>
       </c>
@@ -3794,11 +3936,12 @@
       <c r="C157" t="s">
         <v>281</v>
       </c>
-      <c r="D157">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D157" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E157" s="1"/>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>9209</v>
       </c>
@@ -3808,11 +3951,12 @@
       <c r="C158" t="s">
         <v>283</v>
       </c>
-      <c r="D158">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D158" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E158" s="1"/>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>9210</v>
       </c>
@@ -3822,11 +3966,12 @@
       <c r="C159" t="s">
         <v>284</v>
       </c>
-      <c r="D159">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D159" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E159" s="1"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>9211</v>
       </c>
@@ -3836,9 +3981,10 @@
       <c r="C160" t="s">
         <v>285</v>
       </c>
-      <c r="D160">
-        <v>41640</v>
-      </c>
+      <c r="D160" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E160" s="1"/>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161">
@@ -3850,9 +3996,10 @@
       <c r="C161" t="s">
         <v>286</v>
       </c>
-      <c r="D161">
-        <v>41640</v>
-      </c>
+      <c r="D161" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E161" s="1"/>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162">
@@ -3864,9 +4011,10 @@
       <c r="C162" t="s">
         <v>288</v>
       </c>
-      <c r="D162">
-        <v>41640</v>
-      </c>
+      <c r="D162" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E162" s="1"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163">
@@ -3878,9 +4026,10 @@
       <c r="C163" t="s">
         <v>290</v>
       </c>
-      <c r="D163">
-        <v>41640</v>
-      </c>
+      <c r="D163" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E163" s="1"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164">
@@ -3892,9 +4041,10 @@
       <c r="C164" t="s">
         <v>292</v>
       </c>
-      <c r="D164">
-        <v>41640</v>
-      </c>
+      <c r="D164" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E164" s="1"/>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165">
@@ -3906,9 +4056,10 @@
       <c r="C165" t="s">
         <v>294</v>
       </c>
-      <c r="D165">
-        <v>41640</v>
-      </c>
+      <c r="D165" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E165" s="1"/>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166">
@@ -3920,9 +4071,10 @@
       <c r="C166" t="s">
         <v>296</v>
       </c>
-      <c r="D166">
-        <v>41640</v>
-      </c>
+      <c r="D166" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E166" s="1"/>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167">
@@ -3934,9 +4086,10 @@
       <c r="C167" t="s">
         <v>298</v>
       </c>
-      <c r="D167">
-        <v>41640</v>
-      </c>
+      <c r="D167" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E167" s="1"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168">
@@ -3948,10 +4101,10 @@
       <c r="C168" t="s">
         <v>299</v>
       </c>
-      <c r="D168">
-        <v>41640</v>
-      </c>
-      <c r="E168">
+      <c r="D168" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E168" s="1">
         <v>44377</v>
       </c>
     </row>
@@ -3965,9 +4118,10 @@
       <c r="C169" t="s">
         <v>301</v>
       </c>
-      <c r="D169">
-        <v>41640</v>
-      </c>
+      <c r="D169" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E169" s="1"/>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170">
@@ -3979,9 +4133,10 @@
       <c r="C170" t="s">
         <v>303</v>
       </c>
-      <c r="D170">
-        <v>41640</v>
-      </c>
+      <c r="D170" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E170" s="1"/>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171">
@@ -3993,9 +4148,10 @@
       <c r="C171" t="s">
         <v>299</v>
       </c>
-      <c r="D171">
-        <v>41640</v>
-      </c>
+      <c r="D171" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E171" s="1"/>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172">
@@ -4007,9 +4163,10 @@
       <c r="C172" t="s">
         <v>304</v>
       </c>
-      <c r="D172">
-        <v>41640</v>
-      </c>
+      <c r="D172" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E172" s="1"/>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173">
@@ -4021,9 +4178,10 @@
       <c r="C173" t="s">
         <v>305</v>
       </c>
-      <c r="D173">
-        <v>41640</v>
-      </c>
+      <c r="D173" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E173" s="1"/>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174">
@@ -4035,9 +4193,10 @@
       <c r="C174" t="s">
         <v>306</v>
       </c>
-      <c r="D174">
-        <v>41640</v>
-      </c>
+      <c r="D174" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E174" s="1"/>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175">
@@ -4049,9 +4208,10 @@
       <c r="C175" t="s">
         <v>308</v>
       </c>
-      <c r="D175">
-        <v>41640</v>
-      </c>
+      <c r="D175" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E175" s="1"/>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176">
@@ -4063,9 +4223,10 @@
       <c r="C176" t="s">
         <v>310</v>
       </c>
-      <c r="D176">
-        <v>41640</v>
-      </c>
+      <c r="D176" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E176" s="1"/>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177">
@@ -4077,9 +4238,10 @@
       <c r="C177" t="s">
         <v>312</v>
       </c>
-      <c r="D177">
-        <v>41640</v>
-      </c>
+      <c r="D177" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E177" s="1"/>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178">
@@ -4091,9 +4253,10 @@
       <c r="C178" t="s">
         <v>313</v>
       </c>
-      <c r="D178">
-        <v>41640</v>
-      </c>
+      <c r="D178" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E178" s="1"/>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179">
@@ -4105,9 +4268,10 @@
       <c r="C179" t="s">
         <v>315</v>
       </c>
-      <c r="D179">
-        <v>41640</v>
-      </c>
+      <c r="D179" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E179" s="1"/>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180">
@@ -4119,9 +4283,10 @@
       <c r="C180" t="s">
         <v>317</v>
       </c>
-      <c r="D180">
-        <v>41640</v>
-      </c>
+      <c r="D180" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E180" s="1"/>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181">
@@ -4133,9 +4298,10 @@
       <c r="C181" t="s">
         <v>318</v>
       </c>
-      <c r="D181">
-        <v>41640</v>
-      </c>
+      <c r="D181" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E181" s="1"/>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182">
@@ -4147,9 +4313,10 @@
       <c r="C182" t="s">
         <v>319</v>
       </c>
-      <c r="D182">
-        <v>41640</v>
-      </c>
+      <c r="D182" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E182" s="1"/>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183">
@@ -4161,9 +4328,10 @@
       <c r="C183" t="s">
         <v>320</v>
       </c>
-      <c r="D183">
-        <v>41640</v>
-      </c>
+      <c r="D183" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E183" s="1"/>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184">
@@ -4175,9 +4343,10 @@
       <c r="C184" t="s">
         <v>299</v>
       </c>
-      <c r="D184">
-        <v>41640</v>
-      </c>
+      <c r="D184" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E184" s="1"/>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185">
@@ -4189,9 +4358,10 @@
       <c r="C185" t="s">
         <v>322</v>
       </c>
-      <c r="D185">
+      <c r="D185" s="1">
         <v>45474</v>
       </c>
+      <c r="E185" s="1"/>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186">
@@ -4203,9 +4373,10 @@
       <c r="C186" t="s">
         <v>323</v>
       </c>
-      <c r="D186">
-        <v>41640</v>
-      </c>
+      <c r="D186" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E186" s="1"/>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187">
@@ -4217,9 +4388,10 @@
       <c r="C187" t="s">
         <v>324</v>
       </c>
-      <c r="D187">
-        <v>41640</v>
-      </c>
+      <c r="D187" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E187" s="1"/>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188">
@@ -4231,9 +4403,10 @@
       <c r="C188" t="s">
         <v>326</v>
       </c>
-      <c r="D188">
-        <v>41640</v>
-      </c>
+      <c r="D188" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E188" s="1"/>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189">
@@ -4245,9 +4418,10 @@
       <c r="C189" t="s">
         <v>328</v>
       </c>
-      <c r="D189">
+      <c r="D189" s="1">
         <v>43221</v>
       </c>
+      <c r="E189" s="1"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190">
@@ -4259,9 +4433,10 @@
       <c r="C190" t="s">
         <v>330</v>
       </c>
-      <c r="D190">
-        <v>41640</v>
-      </c>
+      <c r="D190" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E190" s="1"/>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191">
@@ -4273,10 +4448,10 @@
       <c r="C191" t="s">
         <v>332</v>
       </c>
-      <c r="D191">
-        <v>41640</v>
-      </c>
-      <c r="E191">
+      <c r="D191" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E191" s="1">
         <v>44408</v>
       </c>
     </row>
@@ -4290,11 +4465,12 @@
       <c r="C192" t="s">
         <v>334</v>
       </c>
-      <c r="D192">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D192" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E192" s="1"/>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>9292</v>
       </c>
@@ -4304,11 +4480,12 @@
       <c r="C193" t="s">
         <v>335</v>
       </c>
-      <c r="D193">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D193" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E193" s="1"/>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>9293</v>
       </c>
@@ -4318,11 +4495,12 @@
       <c r="C194" t="s">
         <v>336</v>
       </c>
-      <c r="D194">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D194" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E194" s="1"/>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>9294</v>
       </c>
@@ -4332,11 +4510,12 @@
       <c r="C195" t="s">
         <v>338</v>
       </c>
-      <c r="D195">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D195" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E195" s="1"/>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>9299</v>
       </c>
@@ -4346,11 +4525,12 @@
       <c r="C196" t="s">
         <v>340</v>
       </c>
-      <c r="D196">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D196" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E196" s="1"/>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>9901</v>
       </c>
@@ -4360,11 +4540,12 @@
       <c r="C197" t="s">
         <v>342</v>
       </c>
-      <c r="D197">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D197" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E197" s="1"/>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>9902</v>
       </c>
@@ -4374,11 +4555,12 @@
       <c r="C198" t="s">
         <v>343</v>
       </c>
-      <c r="D198">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D198" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E198" s="1"/>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>9903</v>
       </c>
@@ -4388,11 +4570,12 @@
       <c r="C199" t="s">
         <v>344</v>
       </c>
-      <c r="D199">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D199" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E199" s="1"/>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>9904</v>
       </c>
@@ -4402,11 +4585,12 @@
       <c r="C200" t="s">
         <v>345</v>
       </c>
-      <c r="D200">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D200" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E200" s="1"/>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>9905</v>
       </c>
@@ -4416,11 +4600,12 @@
       <c r="C201" t="s">
         <v>347</v>
       </c>
-      <c r="D201">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D201" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E201" s="1"/>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>9906</v>
       </c>
@@ -4430,11 +4615,12 @@
       <c r="C202" t="s">
         <v>349</v>
       </c>
-      <c r="D202">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D202" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E202" s="1"/>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>9907</v>
       </c>
@@ -4444,11 +4630,12 @@
       <c r="C203" t="s">
         <v>351</v>
       </c>
-      <c r="D203">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D203" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E203" s="1"/>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>9908</v>
       </c>
@@ -4458,11 +4645,12 @@
       <c r="C204" t="s">
         <v>353</v>
       </c>
-      <c r="D204">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D204" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E204" s="1"/>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>9910</v>
       </c>
@@ -4472,11 +4660,12 @@
       <c r="C205" t="s">
         <v>355</v>
       </c>
-      <c r="D205">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D205" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E205" s="1"/>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>9911</v>
       </c>
@@ -4486,11 +4675,12 @@
       <c r="C206" t="s">
         <v>356</v>
       </c>
-      <c r="D206">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D206" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E206" s="1"/>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>9912</v>
       </c>
@@ -4500,11 +4690,12 @@
       <c r="C207" t="s">
         <v>358</v>
       </c>
-      <c r="D207">
-        <v>41640</v>
-      </c>
-    </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D207" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E207" s="1"/>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>9930</v>
       </c>
@@ -4514,9 +4705,10 @@
       <c r="C208" t="s">
         <v>360</v>
       </c>
-      <c r="D208">
-        <v>41640</v>
-      </c>
+      <c r="D208" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E208" s="1"/>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209">
@@ -4528,9 +4720,10 @@
       <c r="C209" t="s">
         <v>362</v>
       </c>
-      <c r="D209">
-        <v>41640</v>
-      </c>
+      <c r="D209" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E209" s="1"/>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210">
@@ -4542,9 +4735,10 @@
       <c r="C210" t="s">
         <v>364</v>
       </c>
-      <c r="D210">
-        <v>41640</v>
-      </c>
+      <c r="D210" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E210" s="1"/>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211">
@@ -4556,9 +4750,10 @@
       <c r="C211" t="s">
         <v>366</v>
       </c>
-      <c r="D211">
-        <v>41640</v>
-      </c>
+      <c r="D211" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E211" s="1"/>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212">
@@ -4570,9 +4765,10 @@
       <c r="C212" t="s">
         <v>368</v>
       </c>
-      <c r="D212">
-        <v>41640</v>
-      </c>
+      <c r="D212" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E212" s="1"/>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213">
@@ -4584,9 +4780,10 @@
       <c r="C213" t="s">
         <v>369</v>
       </c>
-      <c r="D213">
-        <v>41640</v>
-      </c>
+      <c r="D213" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E213" s="1"/>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214">
@@ -4598,10 +4795,10 @@
       <c r="C214" t="s">
         <v>370</v>
       </c>
-      <c r="D214">
-        <v>41640</v>
-      </c>
-      <c r="E214">
+      <c r="D214" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E214" s="1">
         <v>43769</v>
       </c>
     </row>
@@ -4615,10 +4812,10 @@
       <c r="C215" t="s">
         <v>371</v>
       </c>
-      <c r="D215">
-        <v>41640</v>
-      </c>
-      <c r="E215">
+      <c r="D215" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E215" s="1">
         <v>43769</v>
       </c>
     </row>
@@ -4632,9 +4829,10 @@
       <c r="C216" t="s">
         <v>373</v>
       </c>
-      <c r="D216">
-        <v>41640</v>
-      </c>
+      <c r="D216" s="1">
+        <v>41640</v>
+      </c>
+      <c r="E216" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>